<commit_message>
Add gloves, goggles, boots and update safety percentage logic
</commit_message>
<xml_diff>
--- a/reports/employee_safety.xlsx
+++ b/reports/employee_safety.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,12 @@
       <b val="1"/>
       <color rgb="00C0392B"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E8449"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="5">
@@ -100,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -118,6 +124,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -570,12 +582,12 @@
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -587,7 +599,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>2026-04-14 18:51:24</t>
+          <t>2026-06-30 23:34:48</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -612,12 +624,12 @@
           <t>Construction</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -629,7 +641,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>2026-04-08 15:41:07</t>
+          <t>2026-06-30 23:07:48</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -654,16 +666,16 @@
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
           <t>NOT READY</t>
@@ -671,12 +683,12 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>2026-04-14 18:48:42</t>
+          <t>2026-06-30 23:13:29</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Missing PPE: Helmet, Safety Vest</t>
+          <t>Missing PPE: Safety Vest</t>
         </is>
       </c>
     </row>
@@ -696,12 +708,12 @@
           <t>Electrical</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -713,12 +725,12 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>2026-04-08 15:42:35</t>
+          <t>2026-07-01 17:33:08</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Missing PPE: Helmet, Safety Vest</t>
+          <t>Missing PPE: Helmet, Safety Vest, Gloves, Glasses, Boots</t>
         </is>
       </c>
     </row>

</xml_diff>